<commit_message>
Prepare offline data for LAB013-018 holdout analysis
</commit_message>
<xml_diff>
--- a/fermentation_model/data/mem2026/LAB013-015/LAB013-LAB015-offline-measurements.xlsx
+++ b/fermentation_model/data/mem2026/LAB013-015/LAB013-LAB015-offline-measurements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\claud\Desktop\Universidad\Memoria\Model\pyomo-doe\fermentation_model\data\mem2026\LAB013-015\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2CE677EE-8268-4A4A-83F2-BB71421FC36C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7056557B-B609-41E1-AD0F-89DEDCD89B57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -404,10 +404,10 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>

</xml_diff>